<commit_message>
interim commit- frsmote now works with instantiation and lateron configuration and building
</commit_message>
<xml_diff>
--- a/temp/gridsearch_results.xlsx
+++ b/temp/gridsearch_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP5"/>
+  <dimension ref="A1:AR3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,180 +461,190 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>param_frsmote__instance_ranking_strategy</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>param_frsmote__k_neighbors</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>param_frsmote__lb_implicator_name</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>param_frsmote__lb_owa_method_name</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>param_frsmote__random_state</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>param_frsmote__sampling_strategy</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>param_frsmote__similarity</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>param_frsmote__similarity_tnorm</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>param_frsmote__type</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>param_frsmote__ub_owa_method_name</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>param_frsmote__ub_tnorm_name</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>param_svc__C</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>param_svc__kernel</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>params</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>split0_test_f1</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>split1_test_f1</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>split2_test_f1</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>mean_test_f1</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>std_test_f1</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>rank_test_f1</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>split0_test_accuracy</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>split1_test_accuracy</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>split2_test_accuracy</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>mean_test_accuracy</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>std_test_accuracy</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>rank_test_accuracy</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>split0_test_precision</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>split1_test_precision</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>split2_test_precision</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>mean_test_precision</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>std_test_precision</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>rank_test_precision</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>split0_test_recall</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>split1_test_recall</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>split2_test_recall</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>mean_test_recall</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>std_test_recall</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>rank_test_recall</t>
         </is>
@@ -642,16 +652,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>21.51229127248128</v>
+        <v>8.004519383112589</v>
       </c>
       <c r="B2" t="n">
-        <v>0.227638886778996</v>
+        <v>0.1061283361683141</v>
       </c>
       <c r="C2" t="n">
-        <v>0.03453397750854492</v>
+        <v>0.01022108395894369</v>
       </c>
       <c r="D2" t="n">
-        <v>0.003046223575781399</v>
+        <v>0.001079736551781181</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -659,145 +669,155 @@
       <c r="F2" t="n">
         <v>0.1</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>pos</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
         <v>5</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>lukasiewicz</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>linear</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>42</v>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>gaussian</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>minimum</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>itfrs</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>owafrs</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t>linear</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>minimum</t>
         </is>
       </c>
-      <c r="P2" t="n">
+      <c r="R2" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>rbf</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>{'frsmote__bias_interpolation': False, 'frsmote__gaussian_similarity_sigma': 0.1, 'frsmote__k_neighbors': 5, 'frsmote__lb_implicator_name': 'lukasiewicz', 'frsmote__lb_owa_method_name': 'linear', 'frsmote__random_state': 42, 'frsmote__similarity': 'gaussian', 'frsmote__similarity_tnorm': 'minimum', 'frsmote__type': 'itfrs', 'frsmote__ub_owa_method_name': 'linear', 'frsmote__ub_tnorm_name': 'minimum', 'svc__C': 0.1, 'svc__kernel': 'rbf'}</t>
-        </is>
-      </c>
-      <c r="S2" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0.5454545454545454</v>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>{'frsmote__bias_interpolation': False, 'frsmote__gaussian_similarity_sigma': 0.1, 'frsmote__instance_ranking_strategy': 'pos', 'frsmote__k_neighbors': 5, 'frsmote__lb_implicator_name': 'lukasiewicz', 'frsmote__lb_owa_method_name': 'linear', 'frsmote__random_state': 42, 'frsmote__sampling_strategy': 'auto', 'frsmote__similarity': 'gaussian', 'frsmote__similarity_tnorm': 'minimum', 'frsmote__type': 'owafrs', 'frsmote__ub_owa_method_name': 'linear', 'frsmote__ub_tnorm_name': 'minimum', 'svc__C': 0.1, 'svc__kernel': 'rbf'}</t>
+        </is>
       </c>
       <c r="U2" t="n">
-        <v>0.7567567567567568</v>
+        <v>0.6829268292682927</v>
       </c>
       <c r="V2" t="n">
-        <v>0.6674037674037674</v>
+        <v>0.5581395348837209</v>
       </c>
       <c r="W2" t="n">
-        <v>0.08928994683950285</v>
+        <v>0.7692307692307693</v>
       </c>
       <c r="X2" t="n">
-        <v>4</v>
+        <v>0.6700990444609277</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.88</v>
+        <v>0.08665368371411251</v>
       </c>
       <c r="Z2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0.8633333333333334</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>0.0410960933531265</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>0.5384615384615384</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>0.6521739130434783</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0.5397356266921484</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>0.09128977759907493</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="AN2" t="n">
         <v>0.8</v>
       </c>
-      <c r="AA2" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>0.8633333333333334</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>0.04642796092394706</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>3</v>
-      </c>
-      <c r="AE2" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="AF2" t="n">
-        <v>0.4137931034482759</v>
-      </c>
-      <c r="AG2" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="AH2" t="n">
-        <v>0.5468199233716474</v>
-      </c>
-      <c r="AI2" t="n">
-        <v>0.1036550225785459</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>3</v>
-      </c>
-      <c r="AK2" t="n">
-        <v>0.9333333333333333</v>
-      </c>
-      <c r="AL2" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="AN2" t="n">
-        <v>0.8694444444444445</v>
-      </c>
       <c r="AO2" t="n">
-        <v>0.05457467417885693</v>
+        <v>0.9375</v>
       </c>
       <c r="AP2" t="n">
-        <v>2</v>
+        <v>0.8902777777777778</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>0.06385868851429247</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>21.40557861328125</v>
+        <v>7.538979291915894</v>
       </c>
       <c r="B3" t="n">
-        <v>0.4262851637051486</v>
+        <v>0.1259330685596834</v>
       </c>
       <c r="C3" t="n">
-        <v>0.02955269813537598</v>
+        <v>0.008006731669108072</v>
       </c>
       <c r="D3" t="n">
-        <v>0.004345791892912741</v>
+        <v>0.0003174067020149583</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -805,423 +825,141 @@
       <c r="F3" t="n">
         <v>0.1</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>pos</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
         <v>5</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>lukasiewicz</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>linear</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>42</v>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>gaussian</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
           <t>minimum</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>owafrs</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>linear</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>minimum</t>
         </is>
       </c>
-      <c r="P3" t="n">
+      <c r="R3" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>rbf</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>{'frsmote__bias_interpolation': False, 'frsmote__gaussian_similarity_sigma': 0.1, 'frsmote__k_neighbors': 5, 'frsmote__lb_implicator_name': 'lukasiewicz', 'frsmote__lb_owa_method_name': 'linear', 'frsmote__random_state': 42, 'frsmote__similarity': 'gaussian', 'frsmote__similarity_tnorm': 'minimum', 'frsmote__type': 'owafrs', 'frsmote__ub_owa_method_name': 'linear', 'frsmote__ub_tnorm_name': 'minimum', 'svc__C': 0.1, 'svc__kernel': 'rbf'}</t>
-        </is>
-      </c>
-      <c r="S3" t="n">
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>{'frsmote__bias_interpolation': False, 'frsmote__gaussian_similarity_sigma': 0.1, 'frsmote__instance_ranking_strategy': 'pos', 'frsmote__k_neighbors': 5, 'frsmote__lb_implicator_name': 'lukasiewicz', 'frsmote__lb_owa_method_name': 'linear', 'frsmote__random_state': 42, 'frsmote__sampling_strategy': 'auto', 'frsmote__similarity': 'linear', 'frsmote__similarity_tnorm': 'minimum', 'frsmote__type': 'owafrs', 'frsmote__ub_owa_method_name': 'linear', 'frsmote__ub_tnorm_name': 'minimum', 'svc__C': 0.1, 'svc__kernel': 'rbf'}</t>
+        </is>
+      </c>
+      <c r="U3" t="n">
         <v>0.6829268292682927</v>
       </c>
-      <c r="T3" t="n">
-        <v>0.5581395348837209</v>
-      </c>
-      <c r="U3" t="n">
-        <v>0.7692307692307693</v>
-      </c>
       <c r="V3" t="n">
-        <v>0.6700990444609277</v>
+        <v>0.55</v>
       </c>
       <c r="W3" t="n">
-        <v>0.08665368371411251</v>
+        <v>0.7894736842105263</v>
       </c>
       <c r="X3" t="n">
-        <v>3</v>
+        <v>0.6741335044929396</v>
       </c>
       <c r="Y3" t="n">
+        <v>0.09796224877572089</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA3" t="n">
         <v>0.87</v>
       </c>
-      <c r="Z3" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>0.91</v>
-      </c>
       <c r="AB3" t="n">
-        <v>0.8633333333333334</v>
+        <v>0.82</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.0410960933531265</v>
+        <v>0.92</v>
       </c>
       <c r="AD3" t="n">
-        <v>3</v>
+        <v>0.87</v>
       </c>
       <c r="AE3" t="n">
+        <v>0.04082482904638634</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG3" t="n">
         <v>0.5384615384615384</v>
       </c>
-      <c r="AF3" t="n">
-        <v>0.4285714285714285</v>
-      </c>
-      <c r="AG3" t="n">
-        <v>0.6521739130434783</v>
-      </c>
       <c r="AH3" t="n">
-        <v>0.5397356266921484</v>
+        <v>0.44</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.09128977759907493</v>
+        <v>0.6818181818181818</v>
       </c>
       <c r="AJ3" t="n">
-        <v>4</v>
+        <v>0.5534265734265734</v>
       </c>
       <c r="AK3" t="n">
+        <v>0.09928736901234833</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM3" t="n">
         <v>0.9333333333333333</v>
       </c>
-      <c r="AL3" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AM3" t="n">
+      <c r="AN3" t="n">
+        <v>0.7333333333333333</v>
+      </c>
+      <c r="AO3" t="n">
         <v>0.9375</v>
       </c>
-      <c r="AN3" t="n">
-        <v>0.8902777777777778</v>
-      </c>
-      <c r="AO3" t="n">
-        <v>0.06385868851429247</v>
-      </c>
       <c r="AP3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>20.95360191663106</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.3504934141910799</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.0421284039815267</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.01482430620187731</v>
-      </c>
-      <c r="E4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G4" t="n">
-        <v>5</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>lukasiewicz</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>linear</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>42</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>linear</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>minimum</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>itfrs</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>linear</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>minimum</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>rbf</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>{'frsmote__bias_interpolation': False, 'frsmote__gaussian_similarity_sigma': 0.1, 'frsmote__k_neighbors': 5, 'frsmote__lb_implicator_name': 'lukasiewicz', 'frsmote__lb_owa_method_name': 'linear', 'frsmote__random_state': 42, 'frsmote__similarity': 'linear', 'frsmote__similarity_tnorm': 'minimum', 'frsmote__type': 'itfrs', 'frsmote__ub_owa_method_name': 'linear', 'frsmote__ub_tnorm_name': 'minimum', 'svc__C': 0.1, 'svc__kernel': 'rbf'}</t>
-        </is>
-      </c>
-      <c r="S4" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="T4" t="n">
-        <v>0.5853658536585366</v>
-      </c>
-      <c r="U4" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="V4" t="n">
-        <v>0.684010840108401</v>
-      </c>
-      <c r="W4" t="n">
-        <v>0.08847813085056637</v>
-      </c>
-      <c r="X4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>0.8733333333333334</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>0.04189935029992182</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>0.5185185185185185</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>0.4615384615384616</v>
-      </c>
-      <c r="AG4" t="n">
-        <v>0.7368421052631579</v>
-      </c>
-      <c r="AH4" t="n">
-        <v>0.5722996951067126</v>
-      </c>
-      <c r="AI4" t="n">
-        <v>0.1186516899119197</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>0.9333333333333333</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>0.8694444444444445</v>
-      </c>
-      <c r="AO4" t="n">
-        <v>0.05457467417885693</v>
-      </c>
-      <c r="AP4" t="n">
+        <v>0.8680555555555555</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>0.09527818270079166</v>
+      </c>
+      <c r="AR3" t="n">
         <v>2</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>21.271107117335</v>
-      </c>
-      <c r="B5" t="n">
-        <v>0.104186725544323</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.02600161234537761</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.005306400805689038</v>
-      </c>
-      <c r="E5" t="b">
-        <v>0</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>lukasiewicz</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>linear</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>42</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>linear</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>minimum</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>owafrs</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>linear</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>minimum</t>
-        </is>
-      </c>
-      <c r="P5" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>rbf</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>{'frsmote__bias_interpolation': False, 'frsmote__gaussian_similarity_sigma': 0.1, 'frsmote__k_neighbors': 5, 'frsmote__lb_implicator_name': 'lukasiewicz', 'frsmote__lb_owa_method_name': 'linear', 'frsmote__random_state': 42, 'frsmote__similarity': 'linear', 'frsmote__similarity_tnorm': 'minimum', 'frsmote__type': 'owafrs', 'frsmote__ub_owa_method_name': 'linear', 'frsmote__ub_tnorm_name': 'minimum', 'svc__C': 0.1, 'svc__kernel': 'rbf'}</t>
-        </is>
-      </c>
-      <c r="S5" t="n">
-        <v>0.6829268292682927</v>
-      </c>
-      <c r="T5" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="U5" t="n">
-        <v>0.7894736842105263</v>
-      </c>
-      <c r="V5" t="n">
-        <v>0.6741335044929396</v>
-      </c>
-      <c r="W5" t="n">
-        <v>0.09796224877572089</v>
-      </c>
-      <c r="X5" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>0.87</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>0.87</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>0.04082482904638634</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE5" t="n">
-        <v>0.5384615384615384</v>
-      </c>
-      <c r="AF5" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="AG5" t="n">
-        <v>0.6818181818181818</v>
-      </c>
-      <c r="AH5" t="n">
-        <v>0.5534265734265734</v>
-      </c>
-      <c r="AI5" t="n">
-        <v>0.09928736901234833</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>2</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>0.9333333333333333</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>0.7333333333333333</v>
-      </c>
-      <c r="AM5" t="n">
-        <v>0.9375</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>0.8680555555555555</v>
-      </c>
-      <c r="AO5" t="n">
-        <v>0.09527818270079166</v>
-      </c>
-      <c r="AP5" t="n">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
move KEEL utilities into a folder entitled KEEL
</commit_message>
<xml_diff>
--- a/temp/gridsearch_results.xlsx
+++ b/temp/gridsearch_results.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR3"/>
+  <dimension ref="A1:AS3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,165 +486,170 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>param_frsmote__sampling_ratio</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>param_frsmote__sampling_strategy</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>param_frsmote__similarity</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>param_frsmote__similarity_tnorm</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>param_frsmote__type</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>param_frsmote__ub_owa_method_name</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>param_frsmote__ub_tnorm_name</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>param_svc__C</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>param_svc__kernel</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>params</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>split0_test_f1</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>split1_test_f1</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>split2_test_f1</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>mean_test_f1</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>std_test_f1</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>rank_test_f1</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>split0_test_accuracy</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>split1_test_accuracy</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>split2_test_accuracy</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>mean_test_accuracy</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>std_test_accuracy</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>rank_test_accuracy</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>split0_test_precision</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>split1_test_precision</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>split2_test_precision</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>mean_test_precision</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>std_test_precision</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>rank_test_precision</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>split0_test_recall</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>split1_test_recall</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>split2_test_recall</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>mean_test_recall</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>std_test_recall</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>rank_test_recall</t>
         </is>
@@ -652,16 +657,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>8.004519383112589</v>
+        <v>7.200620810190837</v>
       </c>
       <c r="B2" t="n">
-        <v>0.1061283361683141</v>
+        <v>0.09366542123704519</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01022108395894369</v>
+        <v>0.02823837598164876</v>
       </c>
       <c r="D2" t="n">
-        <v>0.001079736551781181</v>
+        <v>0.003016390355737267</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -690,134 +695,137 @@
       <c r="K2" t="n">
         <v>42</v>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>gaussian</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>minimum</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>owafrs</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>linear</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>minimum</t>
         </is>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>0.1</v>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>rbf</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>{'frsmote__bias_interpolation': False, 'frsmote__gaussian_similarity_sigma': 0.1, 'frsmote__instance_ranking_strategy': 'pos', 'frsmote__k_neighbors': 5, 'frsmote__lb_implicator_name': 'lukasiewicz', 'frsmote__lb_owa_method_name': 'linear', 'frsmote__random_state': 42, 'frsmote__sampling_strategy': 'auto', 'frsmote__similarity': 'gaussian', 'frsmote__similarity_tnorm': 'minimum', 'frsmote__type': 'owafrs', 'frsmote__ub_owa_method_name': 'linear', 'frsmote__ub_tnorm_name': 'minimum', 'svc__C': 0.1, 'svc__kernel': 'rbf'}</t>
-        </is>
-      </c>
-      <c r="U2" t="n">
-        <v>0.6829268292682927</v>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>{'frsmote__bias_interpolation': False, 'frsmote__gaussian_similarity_sigma': 0.1, 'frsmote__instance_ranking_strategy': 'pos', 'frsmote__k_neighbors': 5, 'frsmote__lb_implicator_name': 'lukasiewicz', 'frsmote__lb_owa_method_name': 'linear', 'frsmote__random_state': 42, 'frsmote__sampling_ratio': 1.0, 'frsmote__sampling_strategy': 'auto', 'frsmote__similarity': 'gaussian', 'frsmote__similarity_tnorm': 'minimum', 'frsmote__type': 'owafrs', 'frsmote__ub_owa_method_name': 'linear', 'frsmote__ub_tnorm_name': 'minimum', 'svc__C': 0.1, 'svc__kernel': 'rbf'}</t>
+        </is>
       </c>
       <c r="V2" t="n">
-        <v>0.5581395348837209</v>
+        <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>0.7692307692307693</v>
+        <v>0.125</v>
       </c>
       <c r="X2" t="n">
-        <v>0.6700990444609277</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.08665368371411251</v>
+        <v>0.1157407407407407</v>
       </c>
       <c r="Z2" t="n">
+        <v>0.09095779029809492</v>
+      </c>
+      <c r="AA2" t="n">
         <v>2</v>
       </c>
-      <c r="AA2" t="n">
-        <v>0.87</v>
-      </c>
       <c r="AB2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.91</v>
+        <v>0.86</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.8633333333333334</v>
+        <v>0.86</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.0410960933531265</v>
+        <v>0.8566666666666666</v>
       </c>
       <c r="AF2" t="n">
+        <v>0.004714045207910321</v>
+      </c>
+      <c r="AG2" t="n">
         <v>2</v>
       </c>
-      <c r="AG2" t="n">
-        <v>0.5384615384615384</v>
-      </c>
       <c r="AH2" t="n">
-        <v>0.4285714285714285</v>
+        <v>0</v>
       </c>
       <c r="AI2" t="n">
-        <v>0.6521739130434783</v>
+        <v>1</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.5397356266921484</v>
+        <v>1</v>
       </c>
       <c r="AK2" t="n">
-        <v>0.09128977759907493</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="AL2" t="n">
+        <v>0.4714045207910317</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>0.06666666666666667</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>0.06388888888888888</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>0.0510688230856951</v>
+      </c>
+      <c r="AS2" t="n">
         <v>2</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>0.9333333333333333</v>
-      </c>
-      <c r="AN2" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AO2" t="n">
-        <v>0.9375</v>
-      </c>
-      <c r="AP2" t="n">
-        <v>0.8902777777777778</v>
-      </c>
-      <c r="AQ2" t="n">
-        <v>0.06385868851429247</v>
-      </c>
-      <c r="AR2" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>7.538979291915894</v>
+        <v>7.179173787434896</v>
       </c>
       <c r="B3" t="n">
-        <v>0.1259330685596834</v>
+        <v>0.05964304549432613</v>
       </c>
       <c r="C3" t="n">
-        <v>0.008006731669108072</v>
+        <v>0.03168129920959473</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0003174067020149583</v>
+        <v>0.00239368763394136</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -846,120 +854,123 @@
       <c r="K3" t="n">
         <v>42</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>linear</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>minimum</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>owafrs</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>linear</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>minimum</t>
         </is>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>0.1</v>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>rbf</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>{'frsmote__bias_interpolation': False, 'frsmote__gaussian_similarity_sigma': 0.1, 'frsmote__instance_ranking_strategy': 'pos', 'frsmote__k_neighbors': 5, 'frsmote__lb_implicator_name': 'lukasiewicz', 'frsmote__lb_owa_method_name': 'linear', 'frsmote__random_state': 42, 'frsmote__sampling_strategy': 'auto', 'frsmote__similarity': 'linear', 'frsmote__similarity_tnorm': 'minimum', 'frsmote__type': 'owafrs', 'frsmote__ub_owa_method_name': 'linear', 'frsmote__ub_tnorm_name': 'minimum', 'svc__C': 0.1, 'svc__kernel': 'rbf'}</t>
-        </is>
-      </c>
-      <c r="U3" t="n">
-        <v>0.6829268292682927</v>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>{'frsmote__bias_interpolation': False, 'frsmote__gaussian_similarity_sigma': 0.1, 'frsmote__instance_ranking_strategy': 'pos', 'frsmote__k_neighbors': 5, 'frsmote__lb_implicator_name': 'lukasiewicz', 'frsmote__lb_owa_method_name': 'linear', 'frsmote__random_state': 42, 'frsmote__sampling_ratio': 1.0, 'frsmote__sampling_strategy': 'auto', 'frsmote__similarity': 'linear', 'frsmote__similarity_tnorm': 'minimum', 'frsmote__type': 'owafrs', 'frsmote__ub_owa_method_name': 'linear', 'frsmote__ub_tnorm_name': 'minimum', 'svc__C': 0.1, 'svc__kernel': 'rbf'}</t>
+        </is>
       </c>
       <c r="V3" t="n">
-        <v>0.55</v>
+        <v>0</v>
       </c>
       <c r="W3" t="n">
-        <v>0.7894736842105263</v>
+        <v>0.3157894736842105</v>
       </c>
       <c r="X3" t="n">
-        <v>0.6741335044929396</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.09796224877572089</v>
+        <v>0.1793372319688109</v>
       </c>
       <c r="Z3" t="n">
+        <v>0.1324388908496143</v>
+      </c>
+      <c r="AA3" t="n">
         <v>1</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AB3" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="AC3" t="n">
         <v>0.87</v>
       </c>
-      <c r="AB3" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>0.92</v>
-      </c>
       <c r="AD3" t="n">
-        <v>0.87</v>
+        <v>0.86</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.04082482904638634</v>
+        <v>0.86</v>
       </c>
       <c r="AF3" t="n">
+        <v>0.008164965809277268</v>
+      </c>
+      <c r="AG3" t="n">
         <v>1</v>
       </c>
-      <c r="AG3" t="n">
-        <v>0.5384615384615384</v>
-      </c>
       <c r="AH3" t="n">
-        <v>0.44</v>
+        <v>0</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.6818181818181818</v>
+        <v>0.75</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.5534265734265734</v>
+        <v>1</v>
       </c>
       <c r="AK3" t="n">
-        <v>0.09928736901234833</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="AL3" t="n">
+        <v>0.4249182927993987</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>0.1083333333333333</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>0.08249579113843056</v>
+      </c>
+      <c r="AS3" t="n">
         <v>1</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>0.9333333333333333</v>
-      </c>
-      <c r="AN3" t="n">
-        <v>0.7333333333333333</v>
-      </c>
-      <c r="AO3" t="n">
-        <v>0.9375</v>
-      </c>
-      <c r="AP3" t="n">
-        <v>0.8680555555555555</v>
-      </c>
-      <c r="AQ3" t="n">
-        <v>0.09527818270079166</v>
-      </c>
-      <c r="AR3" t="n">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>